<commit_message>
chore: run 2026-03-25 18:10 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_25_03_2026.xlsx
+++ b/logs/Consolidado_25_03_2026.xlsx
@@ -679,7 +679,7 @@
         <v>14</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
         <v>7</v>
@@ -717,7 +717,7 @@
         <v>7</v>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
@@ -736,7 +736,7 @@
         <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E7" t="n">
         <v>10</v>
@@ -4316,12 +4316,12 @@
       </c>
       <c r="G88" s="3" t="inlineStr">
         <is>
-          <t>8690955</t>
+          <t>7718428</t>
         </is>
       </c>
       <c r="H88" s="3" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>35%</t>
         </is>
       </c>
     </row>
@@ -4359,7 +4359,7 @@
       </c>
       <c r="G89" s="3" t="inlineStr">
         <is>
-          <t>7718428</t>
+          <t>8690955</t>
         </is>
       </c>
       <c r="H89" s="3" t="inlineStr">
@@ -25957,7 +25957,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>7718428</t>
+          <t>8690955</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
@@ -25995,12 +25995,12 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>8690955</t>
+          <t>7718428</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>35%</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">

</xml_diff>